<commit_message>
Classeurs : commentaires sur Membres/Congés/Historique, retrait EmailsCopieSquad
- Commentaires de cellule explicatifs ajoutés sur les feuilles Membres (Compteur
  = graine, DateDernierSuivi non utilisé, Actif Oui/Non...), Congés (1 jour
  entier, chevauchement) et Historique (écrit par le script, format long).
- Feuille Parametres : ligne legacy EmailsCopieSquad retirée (la config mail,
  Cc inclus, vit désormais dans conf-suivi-squad.json). Rôles Dev/PO conservés
  et listes déroulantes (Rôle, Actif, Congés!Membre) intactes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TdrNHGArbx5RHTtYye3ET1
</commit_message>
<xml_diff>
--- a/suiviexploit/suivi_exploitation_exemple.xlsx
+++ b/suiviexploit/suivi_exploitation_exemple.xlsx
@@ -43,23 +43,163 @@
         </d:r>
       </text>
     </comment>
-    <comment ref="C2" authorId="0">
-      <text>
-        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t xml:space="preserve">Legacy : copie (Cc) historique. Préférez la clé 'Cc' dans conf-suivi-squad.json, qui a la priorité.</t>
-        </d:r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <d:author xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">Suivi Exploitation</d:author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">Une ligne par personne. Nom = identifiant (sert aussi à la feuille Congés et à l'Historique).</t>
+        </d:r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">Rôle (liste déroulante = rôles de la feuille Parametres). Une personne = un rôle.</t>
+        </d:r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">Compteur : graine de départ (nombre de suivis déjà faits avant la mise en place). NB_FOIS = Compteur + désignations dans l'Historique. Laisser vide (=0) pour un nouveau.</t>
+        </d:r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">Actif : Oui/Non. Seuls les 'Oui' sont désignables. Désactiver = mettre Non (ne pas supprimer la ligne).</t>
+        </d:r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">E-mail du membre : destinataire du mail quand la personne est désignée.</t>
+        </d:r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">DateDernierSuivi : informatif uniquement. NON utilisé par l'algorithme (tout est dérivé de l'Historique).</t>
+        </d:r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <d:author xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">Suivi Exploitation</d:author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">Début du congé (date). 1 jour = jour entier (pas de demi-journée).</t>
+        </d:r>
+      </text>
+    </comment>
+    <comment ref="A1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">Membre en congé (liste déroulante = noms de la feuille Membres).</t>
+        </d:r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">Fin du congé (incluse). Un congé chevauchant la semaine cible OU le vendredi précédent exclut la personne.</t>
+        </d:r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <d:author xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">Suivi Exploitation</d:author>
+  </authors>
+  <commentList>
+    <comment ref="G1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">Statut : 'Envoyé' (désignation effective, comptée dans NB_FOIS) ou 'ALERTE' (désignation impossible).</t>
+        </d:r>
+      </text>
+    </comment>
+    <comment ref="A1" authorId="0">
+      <text>
+        <d:r xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">ÉCRIT PAR LE SCRIPT — ne pas saisir à la main. Format long : 1 ligne par rôle désigné et par semaine. SemaineLundi = lundi de la semaine concernée.</t>
+        </d:r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>RolesADesigner</t>
   </si>
@@ -71,12 +211,6 @@
   </si>
   <si>
     <t>Dev</t>
-  </si>
-  <si>
-    <t>EmailsCopieSquad</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>PO</t>
@@ -257,16 +391,10 @@
       <c r="A2" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -282,44 +410,44 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>3</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>3</v>
@@ -331,15 +459,15 @@
         <v>3</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>3</v>
@@ -351,15 +479,15 @@
         <v>2</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" s="0" t="s">
         <v>3</v>
@@ -371,18 +499,18 @@
         <v>5</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D6" s="2">
         <v>46168</v>
@@ -391,32 +519,32 @@
         <v>4</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D8" s="2">
         <v>46182</v>
@@ -425,7 +553,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -438,6 +566,7 @@
     </dataValidation>
   </dataValidations>
   <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -448,18 +577,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B2" s="2">
         <v>46202</v>
@@ -475,6 +604,7 @@
     </dataValidation>
   </dataValidations>
   <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -485,28 +615,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2">
@@ -517,13 +647,13 @@
         <v>3</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -531,20 +661,21 @@
         <v>46189</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
   <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -555,13 +686,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert des évolutions du jour (robustesse, protection classeur, docs)
Retour à l'état du matin (37c5c2b) : la version livrée présente un
dysfonctionnement constaté à l'usage. Les trois commits annulés
(6a8a88a, 9f6a1ed, 3024d26) restent disponibles sur la branche
claude/suiviexploit-review-docs-pic2iu pour diagnostic et correction.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SqfumQut46cMRTN2A6XQHF
</commit_message>
<xml_diff>
--- a/suiviexploit/suivi_exploitation_exemple.xlsx
+++ b/suiviexploit/suivi_exploitation_exemple.xlsx
@@ -359,17 +359,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -414,165 +407,156 @@
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1" style="3"/>
-    <col min="2" max="2" width="9.140625" customWidth="1" style="3"/>
-    <col min="3" max="3" width="9.140625" customWidth="1" style="3"/>
-    <col min="4" max="4" width="9.140625" customWidth="1" style="3"/>
-    <col min="5" max="5" width="9.140625" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" customWidth="1" style="3"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="0" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="2">
         <v>46175</v>
       </c>
       <c r="E3" s="0">
         <v>3</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="0" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="2">
         <v>46182</v>
       </c>
       <c r="E4" s="0">
         <v>2</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="0" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <v>46154</v>
       </c>
       <c r="E5" s="0">
         <v>5</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="0" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="2">
         <v>46168</v>
       </c>
       <c r="E6" s="0">
         <v>4</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="0" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="0" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="2">
         <v>46182</v>
       </c>
       <c r="E8" s="0">
         <v>2</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="0" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection insertRows="0" deleteRows="0" formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0" sheet="1"/>
   <dataValidations count="2">
     <dataValidation type="list" sqref="C2:C1000" showErrorMessage="1" errorStyle="stop" errorTitle="Rôle invalide" error="Choisir un rôle défini dans la feuille Parametres.">
       <formula1>Parametres!$A$2:$A$50</formula1>
@@ -690,7 +674,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection autoFilter="0" sheet="1"/>
   <headerFooter/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
@@ -713,7 +696,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection autoFilter="0" sheet="1"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>